<commit_message>
deploy: refresh fluso benchmark site
</commit_message>
<xml_diff>
--- a/fluso-benchmark/generated/artifacts/benchmark-workbook.xlsx
+++ b/fluso-benchmark/generated/artifacts/benchmark-workbook.xlsx
@@ -69,7 +69,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fluso Frontier Benchmark</t>
+          <t xml:space="preserve">Fluso Dev-Harness Tier 2 Benchmark</t>
         </is>
       </c>
     </row>
@@ -320,7 +320,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -414,7 +414,7 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
@@ -431,7 +431,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -525,7 +525,7 @@
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB3" t="inlineStr">
@@ -542,7 +542,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -636,7 +636,7 @@
       </c>
       <c r="AA4" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB4" t="inlineStr">
@@ -653,7 +653,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -747,7 +747,7 @@
       </c>
       <c r="AA5" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB5" t="inlineStr">
@@ -764,7 +764,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -858,7 +858,7 @@
       </c>
       <c r="AA6" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB6" t="inlineStr">
@@ -875,7 +875,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -969,7 +969,7 @@
       </c>
       <c r="AA7" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB7" t="inlineStr">
@@ -986,7 +986,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1080,7 +1080,7 @@
       </c>
       <c r="AA8" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB8" t="inlineStr">
@@ -1097,7 +1097,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1191,7 +1191,7 @@
       </c>
       <c r="AA9" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB9" t="inlineStr">
@@ -1208,7 +1208,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1302,7 +1302,7 @@
       </c>
       <c r="AA10" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB10" t="inlineStr">
@@ -1319,7 +1319,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -1413,7 +1413,7 @@
       </c>
       <c r="AA11" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB11" t="inlineStr">
@@ -1430,7 +1430,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -1524,7 +1524,7 @@
       </c>
       <c r="AA12" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB12" t="inlineStr">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -1635,7 +1635,7 @@
       </c>
       <c r="AA13" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB13" t="inlineStr">
@@ -1652,7 +1652,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -1746,7 +1746,7 @@
       </c>
       <c r="AA14" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB14" t="inlineStr">
@@ -1763,7 +1763,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -1857,7 +1857,7 @@
       </c>
       <c r="AA15" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB15" t="inlineStr">
@@ -1874,7 +1874,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1968,7 +1968,7 @@
       </c>
       <c r="AA16" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB16" t="inlineStr">
@@ -1985,7 +1985,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -2084,7 +2084,7 @@
       </c>
       <c r="AA17" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB17" t="inlineStr">
@@ -2101,7 +2101,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -2195,7 +2195,7 @@
       </c>
       <c r="AA18" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB18" t="inlineStr">
@@ -2212,7 +2212,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -2311,7 +2311,7 @@
       </c>
       <c r="AA19" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB19" t="inlineStr">
@@ -2328,7 +2328,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2422,7 +2422,7 @@
       </c>
       <c r="AA20" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB20" t="inlineStr">
@@ -2439,7 +2439,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2533,7 +2533,7 @@
       </c>
       <c r="AA21" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB21" t="inlineStr">
@@ -2550,7 +2550,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2644,7 +2644,7 @@
       </c>
       <c r="AA22" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB22" t="inlineStr">
@@ -2661,7 +2661,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2755,7 +2755,7 @@
       </c>
       <c r="AA23" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB23" t="inlineStr">
@@ -2772,7 +2772,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2866,7 +2866,7 @@
       </c>
       <c r="AA24" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB24" t="inlineStr">
@@ -2883,7 +2883,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2977,7 +2977,7 @@
       </c>
       <c r="AA25" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB25" t="inlineStr">
@@ -2994,7 +2994,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="AA26" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB26" t="inlineStr">
@@ -3105,7 +3105,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -3199,7 +3199,7 @@
       </c>
       <c r="AA27" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB27" t="inlineStr">
@@ -3216,7 +3216,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -3310,7 +3310,7 @@
       </c>
       <c r="AA28" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB28" t="inlineStr">
@@ -3327,7 +3327,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -3421,7 +3421,7 @@
       </c>
       <c r="AA29" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB29" t="inlineStr">
@@ -3438,7 +3438,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -3532,7 +3532,7 @@
       </c>
       <c r="AA30" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB30" t="inlineStr">
@@ -3549,7 +3549,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -3648,7 +3648,7 @@
       </c>
       <c r="AA31" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB31" t="inlineStr">
@@ -3665,7 +3665,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -3759,7 +3759,7 @@
       </c>
       <c r="AA32" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB32" t="inlineStr">
@@ -3776,7 +3776,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -3870,7 +3870,7 @@
       </c>
       <c r="AA33" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB33" t="inlineStr">
@@ -3887,7 +3887,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -3986,7 +3986,7 @@
       </c>
       <c r="AA34" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB34" t="inlineStr">
@@ -4003,7 +4003,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -4097,7 +4097,7 @@
       </c>
       <c r="AA35" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB35" t="inlineStr">
@@ -4114,7 +4114,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -4208,7 +4208,7 @@
       </c>
       <c r="AA36" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB36" t="inlineStr">
@@ -4225,7 +4225,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -4319,7 +4319,7 @@
       </c>
       <c r="AA37" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB37" t="inlineStr">
@@ -4336,7 +4336,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -4432,7 +4432,7 @@
       </c>
       <c r="AA38" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB38" t="inlineStr">
@@ -4449,7 +4449,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -4543,7 +4543,7 @@
       </c>
       <c r="AA39" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB39" t="inlineStr">
@@ -4560,7 +4560,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -4654,7 +4654,7 @@
       </c>
       <c r="AA40" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB40" t="inlineStr">
@@ -4671,7 +4671,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -4765,7 +4765,7 @@
       </c>
       <c r="AA41" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB41" t="inlineStr">
@@ -4782,7 +4782,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -4876,7 +4876,7 @@
       </c>
       <c r="AA42" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB42" t="inlineStr">
@@ -4893,7 +4893,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -4987,7 +4987,7 @@
       </c>
       <c r="AA43" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB43" t="inlineStr">
@@ -5004,7 +5004,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -5098,7 +5098,7 @@
       </c>
       <c r="AA44" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB44" t="inlineStr">
@@ -5115,7 +5115,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -5209,7 +5209,7 @@
       </c>
       <c r="AA45" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB45" t="inlineStr">
@@ -5226,7 +5226,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -5320,7 +5320,7 @@
       </c>
       <c r="AA46" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB46" t="inlineStr">
@@ -5337,7 +5337,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -5431,7 +5431,7 @@
       </c>
       <c r="AA47" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB47" t="inlineStr">
@@ -5448,7 +5448,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
@@ -5542,7 +5542,7 @@
       </c>
       <c r="AA48" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB48" t="inlineStr">
@@ -5559,7 +5559,7 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -5658,7 +5658,7 @@
       </c>
       <c r="AA49" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB49" t="inlineStr">
@@ -5675,7 +5675,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -5769,7 +5769,7 @@
       </c>
       <c r="AA50" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB50" t="inlineStr">
@@ -5786,7 +5786,7 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -5880,7 +5880,7 @@
       </c>
       <c r="AA51" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB51" t="inlineStr">
@@ -5897,7 +5897,7 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -5996,7 +5996,7 @@
       </c>
       <c r="AA52" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB52" t="inlineStr">
@@ -6013,7 +6013,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -6112,7 +6112,7 @@
       </c>
       <c r="AA53" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB53" t="inlineStr">
@@ -6129,7 +6129,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -6223,7 +6223,7 @@
       </c>
       <c r="AA54" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB54" t="inlineStr">
@@ -6240,7 +6240,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -6334,7 +6334,7 @@
       </c>
       <c r="AA55" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB55" t="inlineStr">
@@ -6351,7 +6351,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -6445,7 +6445,7 @@
       </c>
       <c r="AA56" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB56" t="inlineStr">
@@ -6462,7 +6462,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -6556,7 +6556,7 @@
       </c>
       <c r="AA57" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB57" t="inlineStr">
@@ -6573,7 +6573,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -6667,7 +6667,7 @@
       </c>
       <c r="AA58" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB58" t="inlineStr">
@@ -6684,7 +6684,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -6778,7 +6778,7 @@
       </c>
       <c r="AA59" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB59" t="inlineStr">
@@ -6795,7 +6795,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -6889,7 +6889,7 @@
       </c>
       <c r="AA60" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB60" t="inlineStr">
@@ -6906,7 +6906,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -7000,7 +7000,7 @@
       </c>
       <c r="AA61" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB61" t="inlineStr">
@@ -7017,7 +7017,7 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -7116,7 +7116,7 @@
       </c>
       <c r="AA62" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB62" t="inlineStr">
@@ -7133,7 +7133,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -7227,7 +7227,7 @@
       </c>
       <c r="AA63" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB63" t="inlineStr">
@@ -7244,7 +7244,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -7338,7 +7338,7 @@
       </c>
       <c r="AA64" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB64" t="inlineStr">
@@ -7355,7 +7355,7 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
@@ -7449,7 +7449,7 @@
       </c>
       <c r="AA65" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB65" t="inlineStr">
@@ -7466,7 +7466,7 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -7560,7 +7560,7 @@
       </c>
       <c r="AA66" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB66" t="inlineStr">
@@ -7577,7 +7577,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -7671,7 +7671,7 @@
       </c>
       <c r="AA67" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB67" t="inlineStr">
@@ -7688,7 +7688,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -7782,7 +7782,7 @@
       </c>
       <c r="AA68" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB68" t="inlineStr">
@@ -7799,7 +7799,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -7893,7 +7893,7 @@
       </c>
       <c r="AA69" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB69" t="inlineStr">
@@ -7910,7 +7910,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -8004,7 +8004,7 @@
       </c>
       <c r="AA70" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB70" t="inlineStr">
@@ -8021,7 +8021,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
@@ -8115,7 +8115,7 @@
       </c>
       <c r="AA71" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB71" t="inlineStr">
@@ -8132,7 +8132,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -8226,7 +8226,7 @@
       </c>
       <c r="AA72" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB72" t="inlineStr">
@@ -8243,7 +8243,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -8337,7 +8337,7 @@
       </c>
       <c r="AA73" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB73" t="inlineStr">
@@ -8354,7 +8354,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -8448,7 +8448,7 @@
       </c>
       <c r="AA74" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB74" t="inlineStr">
@@ -8465,7 +8465,7 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
@@ -8559,7 +8559,7 @@
       </c>
       <c r="AA75" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB75" t="inlineStr">
@@ -8576,7 +8576,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -8670,7 +8670,7 @@
       </c>
       <c r="AA76" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB76" t="inlineStr">
@@ -8687,7 +8687,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
@@ -8781,7 +8781,7 @@
       </c>
       <c r="AA77" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB77" t="inlineStr">
@@ -8798,7 +8798,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -8892,7 +8892,7 @@
       </c>
       <c r="AA78" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB78" t="inlineStr">
@@ -8909,7 +8909,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -9003,7 +9003,7 @@
       </c>
       <c r="AA79" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB79" t="inlineStr">
@@ -17439,7 +17439,7 @@
       </c>
       <c r="AA158" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB158" t="inlineStr">
@@ -17550,7 +17550,7 @@
       </c>
       <c r="AA159" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB159" t="inlineStr">
@@ -17661,7 +17661,7 @@
       </c>
       <c r="AA160" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB160" t="inlineStr">
@@ -17772,7 +17772,7 @@
       </c>
       <c r="AA161" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB161" t="inlineStr">
@@ -17883,7 +17883,7 @@
       </c>
       <c r="AA162" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB162" t="inlineStr">
@@ -17999,7 +17999,7 @@
       </c>
       <c r="AA163" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB163" t="inlineStr">
@@ -18115,7 +18115,7 @@
       </c>
       <c r="AA164" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB164" t="inlineStr">
@@ -18231,7 +18231,7 @@
       </c>
       <c r="AA165" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB165" t="inlineStr">
@@ -18342,7 +18342,7 @@
       </c>
       <c r="AA166" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB166" t="inlineStr">
@@ -18458,7 +18458,7 @@
       </c>
       <c r="AA167" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB167" t="inlineStr">
@@ -18569,7 +18569,7 @@
       </c>
       <c r="AA168" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB168" t="inlineStr">
@@ -18680,7 +18680,7 @@
       </c>
       <c r="AA169" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB169" t="inlineStr">
@@ -18791,7 +18791,7 @@
       </c>
       <c r="AA170" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB170" t="inlineStr">
@@ -18902,7 +18902,7 @@
       </c>
       <c r="AA171" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB171" t="inlineStr">
@@ -19013,7 +19013,7 @@
       </c>
       <c r="AA172" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB172" t="inlineStr">
@@ -19124,7 +19124,7 @@
       </c>
       <c r="AA173" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB173" t="inlineStr">
@@ -19235,7 +19235,7 @@
       </c>
       <c r="AA174" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB174" t="inlineStr">
@@ -19351,7 +19351,7 @@
       </c>
       <c r="AA175" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB175" t="inlineStr">
@@ -19462,7 +19462,7 @@
       </c>
       <c r="AA176" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB176" t="inlineStr">
@@ -19573,7 +19573,7 @@
       </c>
       <c r="AA177" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB177" t="inlineStr">
@@ -19684,7 +19684,7 @@
       </c>
       <c r="AA178" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB178" t="inlineStr">
@@ -19795,7 +19795,7 @@
       </c>
       <c r="AA179" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB179" t="inlineStr">
@@ -19906,7 +19906,7 @@
       </c>
       <c r="AA180" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB180" t="inlineStr">
@@ -20017,7 +20017,7 @@
       </c>
       <c r="AA181" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB181" t="inlineStr">
@@ -20128,7 +20128,7 @@
       </c>
       <c r="AA182" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB182" t="inlineStr">
@@ -20239,7 +20239,7 @@
       </c>
       <c r="AA183" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB183" t="inlineStr">
@@ -20350,7 +20350,7 @@
       </c>
       <c r="AA184" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB184" t="inlineStr">
@@ -20461,7 +20461,7 @@
       </c>
       <c r="AA185" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB185" t="inlineStr">
@@ -20572,7 +20572,7 @@
       </c>
       <c r="AA186" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB186" t="inlineStr">
@@ -20688,7 +20688,7 @@
       </c>
       <c r="AA187" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB187" t="inlineStr">
@@ -20804,7 +20804,7 @@
       </c>
       <c r="AA188" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB188" t="inlineStr">
@@ -20920,7 +20920,7 @@
       </c>
       <c r="AA189" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB189" t="inlineStr">
@@ -21031,7 +21031,7 @@
       </c>
       <c r="AA190" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB190" t="inlineStr">
@@ -21142,7 +21142,7 @@
       </c>
       <c r="AA191" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB191" t="inlineStr">
@@ -21253,7 +21253,7 @@
       </c>
       <c r="AA192" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB192" t="inlineStr">
@@ -21364,7 +21364,7 @@
       </c>
       <c r="AA193" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB193" t="inlineStr">
@@ -21475,7 +21475,7 @@
       </c>
       <c r="AA194" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB194" t="inlineStr">
@@ -21586,7 +21586,7 @@
       </c>
       <c r="AA195" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB195" t="inlineStr">
@@ -21697,7 +21697,7 @@
       </c>
       <c r="AA196" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB196" t="inlineStr">
@@ -21808,7 +21808,7 @@
       </c>
       <c r="AA197" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB197" t="inlineStr">
@@ -21919,7 +21919,7 @@
       </c>
       <c r="AA198" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB198" t="inlineStr">
@@ -22030,7 +22030,7 @@
       </c>
       <c r="AA199" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB199" t="inlineStr">
@@ -22141,7 +22141,7 @@
       </c>
       <c r="AA200" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB200" t="inlineStr">
@@ -22252,7 +22252,7 @@
       </c>
       <c r="AA201" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB201" t="inlineStr">
@@ -22363,7 +22363,7 @@
       </c>
       <c r="AA202" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB202" t="inlineStr">
@@ -22474,7 +22474,7 @@
       </c>
       <c r="AA203" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB203" t="inlineStr">
@@ -22585,7 +22585,7 @@
       </c>
       <c r="AA204" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB204" t="inlineStr">
@@ -22701,7 +22701,7 @@
       </c>
       <c r="AA205" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB205" t="inlineStr">
@@ -22812,7 +22812,7 @@
       </c>
       <c r="AA206" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB206" t="inlineStr">
@@ -22923,7 +22923,7 @@
       </c>
       <c r="AA207" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB207" t="inlineStr">
@@ -23034,7 +23034,7 @@
       </c>
       <c r="AA208" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB208" t="inlineStr">
@@ -23150,7 +23150,7 @@
       </c>
       <c r="AA209" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB209" t="inlineStr">
@@ -23261,7 +23261,7 @@
       </c>
       <c r="AA210" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB210" t="inlineStr">
@@ -23372,7 +23372,7 @@
       </c>
       <c r="AA211" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB211" t="inlineStr">
@@ -23483,7 +23483,7 @@
       </c>
       <c r="AA212" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB212" t="inlineStr">
@@ -23594,7 +23594,7 @@
       </c>
       <c r="AA213" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB213" t="inlineStr">
@@ -23705,7 +23705,7 @@
       </c>
       <c r="AA214" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB214" t="inlineStr">
@@ -23816,7 +23816,7 @@
       </c>
       <c r="AA215" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB215" t="inlineStr">
@@ -23927,7 +23927,7 @@
       </c>
       <c r="AA216" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB216" t="inlineStr">
@@ -24038,7 +24038,7 @@
       </c>
       <c r="AA217" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB217" t="inlineStr">
@@ -24149,7 +24149,7 @@
       </c>
       <c r="AA218" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB218" t="inlineStr">
@@ -24260,7 +24260,7 @@
       </c>
       <c r="AA219" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB219" t="inlineStr">
@@ -24371,7 +24371,7 @@
       </c>
       <c r="AA220" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB220" t="inlineStr">
@@ -24482,7 +24482,7 @@
       </c>
       <c r="AA221" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB221" t="inlineStr">
@@ -24593,7 +24593,7 @@
       </c>
       <c r="AA222" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB222" t="inlineStr">
@@ -24704,7 +24704,7 @@
       </c>
       <c r="AA223" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB223" t="inlineStr">
@@ -24820,7 +24820,7 @@
       </c>
       <c r="AA224" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB224" t="inlineStr">
@@ -24931,7 +24931,7 @@
       </c>
       <c r="AA225" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB225" t="inlineStr">
@@ -25042,7 +25042,7 @@
       </c>
       <c r="AA226" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB226" t="inlineStr">
@@ -25153,7 +25153,7 @@
       </c>
       <c r="AA227" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB227" t="inlineStr">
@@ -25261,7 +25261,7 @@
       </c>
       <c r="AA228" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB228" t="inlineStr">
@@ -25372,7 +25372,7 @@
       </c>
       <c r="AA229" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB229" t="inlineStr">
@@ -25480,7 +25480,7 @@
       </c>
       <c r="AA230" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB230" t="inlineStr">
@@ -25591,7 +25591,7 @@
       </c>
       <c r="AA231" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB231" t="inlineStr">
@@ -25702,7 +25702,7 @@
       </c>
       <c r="AA232" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB232" t="inlineStr">
@@ -25813,7 +25813,7 @@
       </c>
       <c r="AA233" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB233" t="inlineStr">
@@ -25924,7 +25924,7 @@
       </c>
       <c r="AA234" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB234" t="inlineStr">
@@ -26035,7 +26035,7 @@
       </c>
       <c r="AA235" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB235" t="inlineStr">
@@ -34360,7 +34360,7 @@
       </c>
       <c r="B314" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C314" t="inlineStr">
@@ -34466,7 +34466,7 @@
       </c>
       <c r="B315" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C315" t="inlineStr">
@@ -34577,7 +34577,7 @@
       </c>
       <c r="B316" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C316" t="inlineStr">
@@ -34683,7 +34683,7 @@
       </c>
       <c r="B317" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C317" t="inlineStr">
@@ -34794,7 +34794,7 @@
       </c>
       <c r="B318" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C318" t="inlineStr">
@@ -34900,7 +34900,7 @@
       </c>
       <c r="B319" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C319" t="inlineStr">
@@ -35006,7 +35006,7 @@
       </c>
       <c r="B320" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C320" t="inlineStr">
@@ -35114,7 +35114,7 @@
       </c>
       <c r="B321" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C321" t="inlineStr">
@@ -35225,7 +35225,7 @@
       </c>
       <c r="B322" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C322" t="inlineStr">
@@ -35331,7 +35331,7 @@
       </c>
       <c r="B323" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C323" t="inlineStr">
@@ -35437,7 +35437,7 @@
       </c>
       <c r="B324" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C324" t="inlineStr">
@@ -35543,7 +35543,7 @@
       </c>
       <c r="B325" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C325" t="inlineStr">
@@ -35649,7 +35649,7 @@
       </c>
       <c r="B326" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C326" t="inlineStr">
@@ -35755,7 +35755,7 @@
       </c>
       <c r="B327" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C327" t="inlineStr">
@@ -35861,7 +35861,7 @@
       </c>
       <c r="B328" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C328" t="inlineStr">
@@ -35967,7 +35967,7 @@
       </c>
       <c r="B329" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C329" t="inlineStr">
@@ -36078,7 +36078,7 @@
       </c>
       <c r="B330" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C330" t="inlineStr">
@@ -36184,7 +36184,7 @@
       </c>
       <c r="B331" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C331" t="inlineStr">
@@ -36295,7 +36295,7 @@
       </c>
       <c r="B332" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C332" t="inlineStr">
@@ -36401,7 +36401,7 @@
       </c>
       <c r="B333" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C333" t="inlineStr">
@@ -36507,7 +36507,7 @@
       </c>
       <c r="B334" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C334" t="inlineStr">
@@ -36613,7 +36613,7 @@
       </c>
       <c r="B335" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C335" t="inlineStr">
@@ -36719,7 +36719,7 @@
       </c>
       <c r="B336" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C336" t="inlineStr">
@@ -36825,7 +36825,7 @@
       </c>
       <c r="B337" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C337" t="inlineStr">
@@ -36931,7 +36931,7 @@
       </c>
       <c r="B338" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C338" t="inlineStr">
@@ -37037,7 +37037,7 @@
       </c>
       <c r="B339" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C339" t="inlineStr">
@@ -37143,7 +37143,7 @@
       </c>
       <c r="B340" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C340" t="inlineStr">
@@ -37249,7 +37249,7 @@
       </c>
       <c r="B341" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C341" t="inlineStr">
@@ -37355,7 +37355,7 @@
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
@@ -37461,7 +37461,7 @@
       </c>
       <c r="B343" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C343" t="inlineStr">
@@ -37572,7 +37572,7 @@
       </c>
       <c r="B344" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C344" t="inlineStr">
@@ -37683,7 +37683,7 @@
       </c>
       <c r="B345" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C345" t="inlineStr">
@@ -37789,7 +37789,7 @@
       </c>
       <c r="B346" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C346" t="inlineStr">
@@ -37900,7 +37900,7 @@
       </c>
       <c r="B347" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C347" t="inlineStr">
@@ -38006,7 +38006,7 @@
       </c>
       <c r="B348" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C348" t="inlineStr">
@@ -38112,7 +38112,7 @@
       </c>
       <c r="B349" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C349" t="inlineStr">
@@ -38218,7 +38218,7 @@
       </c>
       <c r="B350" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C350" t="inlineStr">
@@ -38329,7 +38329,7 @@
       </c>
       <c r="B351" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C351" t="inlineStr">
@@ -38435,7 +38435,7 @@
       </c>
       <c r="B352" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C352" t="inlineStr">
@@ -38541,7 +38541,7 @@
       </c>
       <c r="B353" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C353" t="inlineStr">
@@ -38647,7 +38647,7 @@
       </c>
       <c r="B354" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C354" t="inlineStr">
@@ -38753,7 +38753,7 @@
       </c>
       <c r="B355" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C355" t="inlineStr">
@@ -38859,7 +38859,7 @@
       </c>
       <c r="B356" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C356" t="inlineStr">
@@ -38965,7 +38965,7 @@
       </c>
       <c r="B357" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C357" t="inlineStr">
@@ -39071,7 +39071,7 @@
       </c>
       <c r="B358" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C358" t="inlineStr">
@@ -39177,7 +39177,7 @@
       </c>
       <c r="B359" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C359" t="inlineStr">
@@ -39283,7 +39283,7 @@
       </c>
       <c r="B360" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C360" t="inlineStr">
@@ -39389,7 +39389,7 @@
       </c>
       <c r="B361" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C361" t="inlineStr">
@@ -39495,7 +39495,7 @@
       </c>
       <c r="B362" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C362" t="inlineStr">
@@ -39601,7 +39601,7 @@
       </c>
       <c r="B363" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C363" t="inlineStr">
@@ -39707,7 +39707,7 @@
       </c>
       <c r="B364" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C364" t="inlineStr">
@@ -39813,7 +39813,7 @@
       </c>
       <c r="B365" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C365" t="inlineStr">
@@ -39919,7 +39919,7 @@
       </c>
       <c r="B366" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C366" t="inlineStr">
@@ -40025,7 +40025,7 @@
       </c>
       <c r="B367" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C367" t="inlineStr">
@@ -40131,7 +40131,7 @@
       </c>
       <c r="B368" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C368" t="inlineStr">
@@ -40237,7 +40237,7 @@
       </c>
       <c r="B369" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C369" t="inlineStr">
@@ -40343,7 +40343,7 @@
       </c>
       <c r="B370" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C370" t="inlineStr">
@@ -40449,7 +40449,7 @@
       </c>
       <c r="B371" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C371" t="inlineStr">
@@ -40555,7 +40555,7 @@
       </c>
       <c r="B372" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C372" t="inlineStr">
@@ -40661,7 +40661,7 @@
       </c>
       <c r="B373" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C373" t="inlineStr">
@@ -40767,7 +40767,7 @@
       </c>
       <c r="B374" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C374" t="inlineStr">
@@ -40873,7 +40873,7 @@
       </c>
       <c r="B375" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C375" t="inlineStr">
@@ -40979,7 +40979,7 @@
       </c>
       <c r="B376" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C376" t="inlineStr">
@@ -41085,7 +41085,7 @@
       </c>
       <c r="B377" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C377" t="inlineStr">
@@ -41191,7 +41191,7 @@
       </c>
       <c r="B378" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C378" t="inlineStr">
@@ -41297,7 +41297,7 @@
       </c>
       <c r="B379" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C379" t="inlineStr">
@@ -41403,7 +41403,7 @@
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C380" t="inlineStr">
@@ -41514,7 +41514,7 @@
       </c>
       <c r="B381" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C381" t="inlineStr">
@@ -41620,7 +41620,7 @@
       </c>
       <c r="B382" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C382" t="inlineStr">
@@ -41726,7 +41726,7 @@
       </c>
       <c r="B383" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C383" t="inlineStr">
@@ -41832,7 +41832,7 @@
       </c>
       <c r="B384" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C384" t="inlineStr">
@@ -41938,7 +41938,7 @@
       </c>
       <c r="B385" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C385" t="inlineStr">
@@ -42044,7 +42044,7 @@
       </c>
       <c r="B386" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C386" t="inlineStr">
@@ -42150,7 +42150,7 @@
       </c>
       <c r="B387" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C387" t="inlineStr">
@@ -42256,7 +42256,7 @@
       </c>
       <c r="B388" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C388" t="inlineStr">
@@ -42362,7 +42362,7 @@
       </c>
       <c r="B389" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C389" t="inlineStr">
@@ -42468,7 +42468,7 @@
       </c>
       <c r="B390" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C390" t="inlineStr">
@@ -42574,7 +42574,7 @@
       </c>
       <c r="B391" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C391" t="inlineStr">
@@ -42774,7 +42774,7 @@
       </c>
       <c r="AA392" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB392" t="inlineStr">
@@ -42885,7 +42885,7 @@
       </c>
       <c r="AA393" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB393" t="inlineStr">
@@ -42996,7 +42996,7 @@
       </c>
       <c r="AA394" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB394" t="inlineStr">
@@ -43107,7 +43107,7 @@
       </c>
       <c r="AA395" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB395" t="inlineStr">
@@ -43218,7 +43218,7 @@
       </c>
       <c r="AA396" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB396" t="inlineStr">
@@ -43331,7 +43331,7 @@
       </c>
       <c r="AA397" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB397" t="inlineStr">
@@ -43442,7 +43442,7 @@
       </c>
       <c r="AA398" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB398" t="inlineStr">
@@ -43553,7 +43553,7 @@
       </c>
       <c r="AA399" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB399" t="inlineStr">
@@ -43664,7 +43664,7 @@
       </c>
       <c r="AA400" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB400" t="inlineStr">
@@ -43775,7 +43775,7 @@
       </c>
       <c r="AA401" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB401" t="inlineStr">
@@ -43891,7 +43891,7 @@
       </c>
       <c r="AA402" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB402" t="inlineStr">
@@ -44002,7 +44002,7 @@
       </c>
       <c r="AA403" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB403" t="inlineStr">
@@ -44113,7 +44113,7 @@
       </c>
       <c r="AA404" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB404" t="inlineStr">
@@ -44224,7 +44224,7 @@
       </c>
       <c r="AA405" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB405" t="inlineStr">
@@ -44335,7 +44335,7 @@
       </c>
       <c r="AA406" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB406" t="inlineStr">
@@ -44446,7 +44446,7 @@
       </c>
       <c r="AA407" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB407" t="inlineStr">
@@ -44562,7 +44562,7 @@
       </c>
       <c r="AA408" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB408" t="inlineStr">
@@ -44678,7 +44678,7 @@
       </c>
       <c r="AA409" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB409" t="inlineStr">
@@ -44789,7 +44789,7 @@
       </c>
       <c r="AA410" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB410" t="inlineStr">
@@ -44900,7 +44900,7 @@
       </c>
       <c r="AA411" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB411" t="inlineStr">
@@ -45011,7 +45011,7 @@
       </c>
       <c r="AA412" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB412" t="inlineStr">
@@ -45122,7 +45122,7 @@
       </c>
       <c r="AA413" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB413" t="inlineStr">
@@ -45233,7 +45233,7 @@
       </c>
       <c r="AA414" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB414" t="inlineStr">
@@ -45344,7 +45344,7 @@
       </c>
       <c r="AA415" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB415" t="inlineStr">
@@ -45455,7 +45455,7 @@
       </c>
       <c r="AA416" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB416" t="inlineStr">
@@ -45566,7 +45566,7 @@
       </c>
       <c r="AA417" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB417" t="inlineStr">
@@ -45677,7 +45677,7 @@
       </c>
       <c r="AA418" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB418" t="inlineStr">
@@ -45788,7 +45788,7 @@
       </c>
       <c r="AA419" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB419" t="inlineStr">
@@ -45899,7 +45899,7 @@
       </c>
       <c r="AA420" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB420" t="inlineStr">
@@ -46015,7 +46015,7 @@
       </c>
       <c r="AA421" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB421" t="inlineStr">
@@ -46126,7 +46126,7 @@
       </c>
       <c r="AA422" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB422" t="inlineStr">
@@ -46237,7 +46237,7 @@
       </c>
       <c r="AA423" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB423" t="inlineStr">
@@ -46348,7 +46348,7 @@
       </c>
       <c r="AA424" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB424" t="inlineStr">
@@ -46459,7 +46459,7 @@
       </c>
       <c r="AA425" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB425" t="inlineStr">
@@ -46570,7 +46570,7 @@
       </c>
       <c r="AA426" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB426" t="inlineStr">
@@ -46681,7 +46681,7 @@
       </c>
       <c r="AA427" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB427" t="inlineStr">
@@ -46792,7 +46792,7 @@
       </c>
       <c r="AA428" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB428" t="inlineStr">
@@ -46903,7 +46903,7 @@
       </c>
       <c r="AA429" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB429" t="inlineStr">
@@ -47014,7 +47014,7 @@
       </c>
       <c r="AA430" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB430" t="inlineStr">
@@ -47125,7 +47125,7 @@
       </c>
       <c r="AA431" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB431" t="inlineStr">
@@ -47236,7 +47236,7 @@
       </c>
       <c r="AA432" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB432" t="inlineStr">
@@ -47347,7 +47347,7 @@
       </c>
       <c r="AA433" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB433" t="inlineStr">
@@ -47458,7 +47458,7 @@
       </c>
       <c r="AA434" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB434" t="inlineStr">
@@ -47569,7 +47569,7 @@
       </c>
       <c r="AA435" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB435" t="inlineStr">
@@ -47680,7 +47680,7 @@
       </c>
       <c r="AA436" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB436" t="inlineStr">
@@ -47791,7 +47791,7 @@
       </c>
       <c r="AA437" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB437" t="inlineStr">
@@ -47902,7 +47902,7 @@
       </c>
       <c r="AA438" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB438" t="inlineStr">
@@ -48013,7 +48013,7 @@
       </c>
       <c r="AA439" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB439" t="inlineStr">
@@ -48129,7 +48129,7 @@
       </c>
       <c r="AA440" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB440" t="inlineStr">
@@ -48240,7 +48240,7 @@
       </c>
       <c r="AA441" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB441" t="inlineStr">
@@ -48356,7 +48356,7 @@
       </c>
       <c r="AA442" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB442" t="inlineStr">
@@ -48467,7 +48467,7 @@
       </c>
       <c r="AA443" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB443" t="inlineStr">
@@ -48578,7 +48578,7 @@
       </c>
       <c r="AA444" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB444" t="inlineStr">
@@ -48689,7 +48689,7 @@
       </c>
       <c r="AA445" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB445" t="inlineStr">
@@ -48800,7 +48800,7 @@
       </c>
       <c r="AA446" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB446" t="inlineStr">
@@ -48911,7 +48911,7 @@
       </c>
       <c r="AA447" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB447" t="inlineStr">
@@ -49022,7 +49022,7 @@
       </c>
       <c r="AA448" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB448" t="inlineStr">
@@ -49133,7 +49133,7 @@
       </c>
       <c r="AA449" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB449" t="inlineStr">
@@ -49244,7 +49244,7 @@
       </c>
       <c r="AA450" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB450" t="inlineStr">
@@ -49355,7 +49355,7 @@
       </c>
       <c r="AA451" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB451" t="inlineStr">
@@ -49466,7 +49466,7 @@
       </c>
       <c r="AA452" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB452" t="inlineStr">
@@ -49577,7 +49577,7 @@
       </c>
       <c r="AA453" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB453" t="inlineStr">
@@ -49688,7 +49688,7 @@
       </c>
       <c r="AA454" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB454" t="inlineStr">
@@ -49799,7 +49799,7 @@
       </c>
       <c r="AA455" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB455" t="inlineStr">
@@ -49910,7 +49910,7 @@
       </c>
       <c r="AA456" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB456" t="inlineStr">
@@ -50021,7 +50021,7 @@
       </c>
       <c r="AA457" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB457" t="inlineStr">
@@ -50132,7 +50132,7 @@
       </c>
       <c r="AA458" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB458" t="inlineStr">
@@ -50243,7 +50243,7 @@
       </c>
       <c r="AA459" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB459" t="inlineStr">
@@ -50354,7 +50354,7 @@
       </c>
       <c r="AA460" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB460" t="inlineStr">
@@ -50465,7 +50465,7 @@
       </c>
       <c r="AA461" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB461" t="inlineStr">
@@ -50578,7 +50578,7 @@
       </c>
       <c r="AA462" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB462" t="inlineStr">
@@ -50689,7 +50689,7 @@
       </c>
       <c r="AA463" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB463" t="inlineStr">
@@ -50800,7 +50800,7 @@
       </c>
       <c r="AA464" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB464" t="inlineStr">
@@ -50911,7 +50911,7 @@
       </c>
       <c r="AA465" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB465" t="inlineStr">
@@ -51022,7 +51022,7 @@
       </c>
       <c r="AA466" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB466" t="inlineStr">
@@ -51133,7 +51133,7 @@
       </c>
       <c r="AA467" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB467" t="inlineStr">
@@ -51244,7 +51244,7 @@
       </c>
       <c r="AA468" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB468" t="inlineStr">
@@ -51355,7 +51355,7 @@
       </c>
       <c r="AA469" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="AB469" t="inlineStr">
@@ -51446,7 +51446,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t xml:space="preserve">GLM 5.1</t>
+          <t xml:space="preserve">GLM-5.1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -51456,7 +51456,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="E2" t="b">
@@ -51554,7 +51554,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="E4" t="b">
@@ -51642,7 +51642,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gemini 3.1 Pro</t>
+          <t xml:space="preserve">Gemini 3.1 Pro Preview</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -51701,7 +51701,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t xml:space="preserve">valid</t>
+          <t xml:space="preserve">invalid</t>
         </is>
       </c>
       <c r="E7" t="b">

</xml_diff>